<commit_message>
updated answers to be more accurate
</commit_message>
<xml_diff>
--- a/eval/results/answers/agent-a.xlsx
+++ b/eval/results/answers/agent-a.xlsx
@@ -568,7 +568,11 @@
 Answer: The standard game supports 2 to 5 players. The rulebook also mentions additional rules for other game variants on page 13, which I did not check, so I can't say from these excerpts what counts there.</t>
         </is>
       </c>
-      <c r="F2" s="1" t="n"/>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
       <c r="G2" s="1" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
@@ -635,7 +639,11 @@
 Answer: The maximum number of players in the standard game is 5.</t>
         </is>
       </c>
-      <c r="F3" s="1" t="n"/>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G3" s="1" t="n"/>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
@@ -703,7 +711,11 @@
 Answer: The game includes 9 ocean tiles. The board also has 12 reserved ocean areas, but those are board spaces, not tiles.</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n"/>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G4" s="1" t="n"/>
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="n"/>
@@ -770,7 +782,11 @@
 Answer: 12 areas are reserved for ocean tiles.</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n"/>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G5" s="1" t="n"/>
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
@@ -837,7 +853,11 @@
 Answer: The game ends at the end of the generation in which all three global parameters (ocean, temperature, and oxygen) reach their goals. That generation finishes after the production phase, and players then get one extra chance to convert plants into greenery tiles, after which final scoring takes place.</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n"/>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G6" s="1" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="n"/>
@@ -904,7 +924,11 @@
 Answer: Buying a card into your hand during the research phase costs 3 M€ each. This is the buying cost only; the cost to play a card from your hand is a separate amount shown in the card's upper left corner [Terraforming Mars p.6].</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n"/>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G7" s="1" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
@@ -971,7 +995,11 @@
 Answer: No. Temperature and oxygen stop at their maximum goal (temperature at 8°C, oxygen at 14%). Once a parameter reaches its goal, it cannot be raised further. You can still play cards or use actions that raise it, but you ignore that part of the effect, and it does not increase your TR.</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n"/>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G8" s="1" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
@@ -1039,7 +1067,11 @@
 Answer: Yes, but only through cards that show a red border on the resource or production symbol. Those cards can target any player, including an opponent. Cards without a red border always affect only yourself. Also, if a red-bordered production reduction can't be fully applied to the opponent, you must lower your own production or not play the card.</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n"/>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G9" s="1" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
@@ -1106,7 +1138,11 @@
 Answer: The game's resources are twigs, resin, pebbles, and berries. The components list gives 30 twigs, 25 resin, 20 pebbles, and 30 berries. The rulebook does not explicitly label these as the "main" resources, but they are the four resource types set out in the setup.</t>
         </is>
       </c>
-      <c r="F10" s="1" t="n"/>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G10" s="1" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
@@ -1173,7 +1209,11 @@
 Answer: You prepare for the next season on your turn, once you have placed all of your workers and either cannot play a card or do not wish to. You then bring back all your deployed workers and gain the listed bonuses for the next season, shown atop the Ever Tree. Your turn then ends.</t>
         </is>
       </c>
-      <c r="F11" s="1" t="n"/>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
@@ -1240,7 +1280,11 @@
 Answer: You can have up to 15 cards in your city. Event cards do not count toward this limit.</t>
         </is>
       </c>
-      <c r="F12" s="1" t="n"/>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G12" s="1" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
@@ -1307,7 +1351,11 @@
 Answer: An exclusive location can hold only 1 worker, while a shared location can hold multiple workers, even of the same color. Shared locations are shown with an open encircling ring.</t>
         </is>
       </c>
-      <c r="F13" s="1" t="n"/>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G13" s="1" t="n"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
@@ -1374,8 +1422,16 @@
 Answer: Yes, resources can run out. The rules say that if any resources run out, you should use something else as a substitute. The rulebook does not say what to use as a substitute for a specific resource, so that is left to the players.</t>
         </is>
       </c>
-      <c r="F14" s="1" t="n"/>
-      <c r="G14" s="1" t="n"/>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
@@ -1441,7 +1497,11 @@
 Answer: A 4-player game uses 1 Sheriff, 1 Renegade, and 2 Outlaws. There are no Deputies in a 4-player game.</t>
         </is>
       </c>
-      <c r="F15" s="1" t="n"/>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G15" s="1" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
@@ -1508,7 +1568,11 @@
 Answer: Panic! can be played on a player at distance 1. That distance is not changed by weapons, only by cards such as Mustang and/or Scope.</t>
         </is>
       </c>
-      <c r="F16" s="1" t="n"/>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G16" s="1" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
@@ -1576,7 +1640,11 @@
 Answer: With your own Mustang, you still see other players at normal distance, so Panic! works on players at distance 1 from you. The Mustang does not let you reach farther with Panic!, since it only makes other players see you at a greater distance. The Panic! rule text also says Mustang can modify this distance, which seems to conflict with the Mustang's own text, so the rulebook is not fully clear on this point.</t>
         </is>
       </c>
-      <c r="F17" s="1" t="n"/>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G17" s="1" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
@@ -1643,7 +1711,11 @@
 Answer: Panic! still targets a player at distance 1, but with Scope in play you see other players at a distance decreased by 1. So with Scope you can play Panic! on any player who is at actual distance 2 from you (they count as distance 1). Players at distance 1 are still valid, and since distances less than 1 count as 1, the minimum is still 1.</t>
         </is>
       </c>
-      <c r="F18" s="1" t="n"/>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G18" s="1" t="n"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
@@ -1710,7 +1782,11 @@
 Answer: Dynamite is checked first, before the Jail. If you are in jail and have Dynamite in play, you resolve the Dynamite "draw!" at the start of your turn before the jail draw. The rulebook excerpts do not say what happens to the jail draw if the Dynamite explodes or passes, so that is not covered.</t>
         </is>
       </c>
-      <c r="F19" s="1" t="n"/>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G19" s="1" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
@@ -1777,7 +1853,11 @@
 Answer: El Gringo and Paul Regret are the only characters listed with 3 life points.</t>
         </is>
       </c>
-      <c r="F20" s="1" t="n"/>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G20" s="1" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="n"/>
@@ -1845,7 +1925,11 @@
 Answer: Against Slab the Killer, a successful Barrel counts as only one Missed!, so you still need a second defence to cancel his BANG!. Use the Barrel first; if it succeeds (a Heart), you still need to play one Missed! card from your hand to cancel the shot. If the Barrel fails, you need to play two Missed! cards. The rules do not say what happens if you have no second Missed! available.</t>
         </is>
       </c>
-      <c r="F21" s="1" t="n"/>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G21" s="1" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
@@ -1912,8 +1996,16 @@
 Answer: Yes. The dynamite deals 3 damage, and each Beer restores 1 life point. From 1 life, you would need 3 Beers to end at 1 life (1-3+3), since the rulebook's own example shows that each Beer counts for one point. Two Beers would leave you at 0 and eliminated. Beers do nothing if only 2 players remain. The rules also say a Beer can be played out of turn only after a lethal hit, and a dynamite explosion happens at the start of your turn, so you would play the Beers during your turn. The excerpts don't say whether a dynamite hit counts as a lethal hit for out-of-turn play, so I can't confirm that point.</t>
         </is>
       </c>
-      <c r="F22" s="1" t="n"/>
-      <c r="G22" s="1" t="n"/>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="inlineStr">
@@ -1979,7 +2071,11 @@
 Answer: The excerpts don't describe any general trading between players. The only time cards pass to another player is when a card's effect requires it, such as a Critter that says to give the other card to an opponent. In that case you choose an opponent with room in their hand.</t>
         </is>
       </c>
-      <c r="F23" s="1" t="n"/>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G23" s="1" t="n"/>
       <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="n"/>
@@ -2044,7 +2140,11 @@
 Answer: The rules do not name a single best corporation for beginners. The closest guidance is that new players can use the Beginner corporation instead of choosing one of the unique corporations. It starts with 42 MegaCredits and lets the player keep all 10 project cards, and it is "typically used for players new to the game." The rules do not rank any of the unique corporations as the best choice for beginners.</t>
         </is>
       </c>
-      <c r="F24" s="1" t="n"/>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G24" s="1" t="n"/>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
@@ -2111,7 +2211,11 @@
 Answer: not in the rules</t>
         </is>
       </c>
-      <c r="F25" s="1" t="n"/>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>correct</t>
+        </is>
+      </c>
       <c r="G25" s="1" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>

</xml_diff>